<commit_message>
Sync FEC rebuild: Cast & Crew List live in the compiled bundle
Verified byte-identical against ce0ceeb before syncing: decoded
__OM_EMBEDDED_MODULE_SOURCE__ and the text/x-dc app-logic block from
the delivered index.html and diffed both against the exact committed
source (CRLF-normalized) -- exact match. __OM_EMBEDDED_WORKBOOKS__
carries all 4 keys, __OM_EMBEDDED_MODULE_SOURCE__ carries 1, per the
usual two markers.

Also updates the bundled default texas.xlsx to the current published
template (MAY 2026 2.1, with the Cast & Crew List "From Documents"
column) -- byte-identical to Steven's own Templates/ copy -- so a
fresh/bundled-only run gets Cast & Crew List (and the 4-column TX
Crew Payroll layout) without needing a separate Publish/Replace.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source/assets/workbooks/texas.xlsx
+++ b/source/assets/workbooks/texas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tpcus808.sharepoint.com/sites/DataEntryAutomation/Shared Documents/New Automation Documents/Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_F04EF44A1142426DCE9F4511414016BFA20E4AD1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8555807C-BFC7-45DE-B4A1-AF3E07847AD8}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="11_F04EF44A1142426DCE9F4511414016BFA20E4AD1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5A90798-1D72-4250-8B23-D7712328D52A}"/>
   <bookViews>
-    <workbookView xWindow="330" yWindow="435" windowWidth="21600" windowHeight="12450" tabRatio="851" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-11856" yWindow="12852" windowWidth="23256" windowHeight="13896" tabRatio="851" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -185,7 +185,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="304">
   <si>
     <t>35% of paid crew must be Texas Residents</t>
   </si>
@@ -787,36 +787,15 @@
     <t>1st Shoot date</t>
   </si>
   <si>
-    <t>CREW #1</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
     <t>120 Days Prior to Shoot date</t>
   </si>
   <si>
-    <t>CREW #2</t>
-  </si>
-  <si>
     <t>TOTAL TX ONLY - CREW &amp; CAST</t>
   </si>
   <si>
     <t>TOTAL ALL CREW &amp; CAST</t>
   </si>
   <si>
-    <t>CAST #1</t>
-  </si>
-  <si>
-    <t>CAST #2</t>
-  </si>
-  <si>
-    <t>CAST #3</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
     <t>Pay period to Check Number</t>
   </si>
   <si>
@@ -1115,6 +1094,9 @@
   </si>
   <si>
     <t>On PTIP</t>
+  </si>
+  <si>
+    <t>From Documents</t>
   </si>
 </sst>
 </file>
@@ -2692,16 +2674,40 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -2713,37 +2719,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2754,6 +2730,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="11">
@@ -3263,13 +3245,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
@@ -3340,28 +3315,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3396,6 +3350,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
@@ -3418,6 +3379,27 @@
       <fill>
         <patternFill>
           <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3452,6 +3434,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="3" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
@@ -3460,6 +3449,48 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3515,41 +3546,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
@@ -3592,21 +3588,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor theme="3" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3627,14 +3609,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF00B050"/>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3795,34 +3777,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
@@ -3879,6 +3833,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
@@ -3893,6 +3854,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
@@ -3901,6 +3869,20 @@
       <fill>
         <patternFill>
           <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3991,14 +3973,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF00B050"/>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4089,21 +4071,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="3" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4138,6 +4106,20 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
@@ -4152,14 +4134,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF00B050"/>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4488,40 +4470,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="121" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="404" t="s">
+      <c r="A1" s="397" t="s">
         <v>63</v>
       </c>
-      <c r="B1" s="405"/>
-      <c r="C1" s="405"/>
-      <c r="D1" s="405"/>
-      <c r="E1" s="405"/>
-      <c r="F1" s="405"/>
-      <c r="G1" s="405"/>
-      <c r="H1" s="405"/>
-      <c r="I1" s="405"/>
-      <c r="J1" s="405"/>
-      <c r="K1" s="405"/>
-      <c r="L1" s="405"/>
-      <c r="M1" s="405"/>
-      <c r="N1" s="405"/>
+      <c r="B1" s="398"/>
+      <c r="C1" s="398"/>
+      <c r="D1" s="398"/>
+      <c r="E1" s="398"/>
+      <c r="F1" s="398"/>
+      <c r="G1" s="398"/>
+      <c r="H1" s="398"/>
+      <c r="I1" s="398"/>
+      <c r="J1" s="398"/>
+      <c r="K1" s="398"/>
+      <c r="L1" s="398"/>
+      <c r="M1" s="398"/>
+      <c r="N1" s="398"/>
     </row>
     <row r="2" spans="1:15" s="121" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="404" t="s">
+      <c r="A2" s="397" t="s">
         <v>64</v>
       </c>
-      <c r="B2" s="405"/>
-      <c r="C2" s="405"/>
-      <c r="D2" s="405"/>
-      <c r="E2" s="405"/>
-      <c r="F2" s="405"/>
-      <c r="G2" s="405"/>
-      <c r="H2" s="405"/>
-      <c r="I2" s="405"/>
-      <c r="J2" s="405"/>
-      <c r="K2" s="405"/>
-      <c r="L2" s="405"/>
-      <c r="M2" s="405"/>
-      <c r="N2" s="405"/>
+      <c r="B2" s="398"/>
+      <c r="C2" s="398"/>
+      <c r="D2" s="398"/>
+      <c r="E2" s="398"/>
+      <c r="F2" s="398"/>
+      <c r="G2" s="398"/>
+      <c r="H2" s="398"/>
+      <c r="I2" s="398"/>
+      <c r="J2" s="398"/>
+      <c r="K2" s="398"/>
+      <c r="L2" s="398"/>
+      <c r="M2" s="398"/>
+      <c r="N2" s="398"/>
     </row>
     <row r="4" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="229"/>
@@ -4609,12 +4591,12 @@
       </c>
       <c r="D9" s="229"/>
       <c r="E9" s="229"/>
-      <c r="G9" s="406" t="s">
+      <c r="G9" s="399" t="s">
         <v>72</v>
       </c>
-      <c r="H9" s="407"/>
-      <c r="I9" s="407"/>
-      <c r="J9" s="407"/>
+      <c r="H9" s="396"/>
+      <c r="I9" s="396"/>
+      <c r="J9" s="396"/>
       <c r="K9" s="229"/>
       <c r="L9" s="229"/>
       <c r="M9" s="229"/>
@@ -5378,10 +5360,10 @@
       <c r="N43" s="229"/>
     </row>
     <row r="44" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="C44" s="408" t="s">
+      <c r="C44" s="395" t="s">
         <v>131</v>
       </c>
-      <c r="D44" s="407"/>
+      <c r="D44" s="396"/>
       <c r="E44" s="320" t="b">
         <v>0</v>
       </c>
@@ -5391,10 +5373,10 @@
       <c r="N44" s="229"/>
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="C45" s="408" t="s">
+      <c r="C45" s="395" t="s">
         <v>132</v>
       </c>
-      <c r="D45" s="407"/>
+      <c r="D45" s="396"/>
       <c r="E45" s="320" t="b">
         <v>0</v>
       </c>
@@ -5404,10 +5386,10 @@
       <c r="N45" s="229"/>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="C46" s="408" t="s">
+      <c r="C46" s="395" t="s">
         <v>133</v>
       </c>
-      <c r="D46" s="407"/>
+      <c r="D46" s="396"/>
       <c r="E46" s="320" t="b">
         <v>0</v>
       </c>
@@ -5417,10 +5399,10 @@
       <c r="N46" s="229"/>
     </row>
     <row r="47" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="C47" s="408" t="s">
+      <c r="C47" s="395" t="s">
         <v>134</v>
       </c>
-      <c r="D47" s="407"/>
+      <c r="D47" s="396"/>
       <c r="E47" s="320" t="b">
         <v>0</v>
       </c>
@@ -5430,10 +5412,10 @@
       <c r="N47" s="229"/>
     </row>
     <row r="48" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="C48" s="408" t="s">
+      <c r="C48" s="395" t="s">
         <v>135</v>
       </c>
-      <c r="D48" s="407"/>
+      <c r="D48" s="396"/>
       <c r="E48" s="320" t="b">
         <v>0</v>
       </c>
@@ -5443,10 +5425,10 @@
       <c r="N48" s="229"/>
     </row>
     <row r="49" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C49" s="408" t="s">
+      <c r="C49" s="395" t="s">
         <v>136</v>
       </c>
-      <c r="D49" s="407"/>
+      <c r="D49" s="396"/>
       <c r="E49" s="320" t="b">
         <v>0</v>
       </c>
@@ -5455,10 +5437,10 @@
       <c r="M49" s="229"/>
     </row>
     <row r="50" spans="3:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C50" s="409" t="s">
+      <c r="C50" s="393" t="s">
         <v>137</v>
       </c>
-      <c r="D50" s="410"/>
+      <c r="D50" s="394"/>
       <c r="E50" s="321" t="b">
         <v>0</v>
       </c>
@@ -5551,8 +5533,8 @@
         <v>144</v>
       </c>
       <c r="E62" s="324">
-        <f>'Cast &amp; Crew List'!K8</f>
-        <v>5</v>
+        <f>'Cast &amp; Crew List'!L8</f>
+        <v>0</v>
       </c>
     </row>
     <row r="63" spans="3:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -5561,8 +5543,8 @@
         <v>145</v>
       </c>
       <c r="E63" s="326">
-        <f>'Cast &amp; Crew List'!K7</f>
-        <v>4</v>
+        <f>'Cast &amp; Crew List'!L7</f>
+        <v>0</v>
       </c>
     </row>
     <row r="64" spans="3:13" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
@@ -5570,9 +5552,9 @@
       <c r="D64" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="E64" s="327">
+      <c r="E64" s="327" t="e">
         <f>E63/E62</f>
-        <v>0.8</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="65" spans="3:5" x14ac:dyDescent="0.3">
@@ -5589,16 +5571,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="G9:J9"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="A2:N2"/>
     <mergeCell ref="C50:D50"/>
     <mergeCell ref="C45:D45"/>
     <mergeCell ref="C44:D44"/>
     <mergeCell ref="C48:D48"/>
     <mergeCell ref="C49:D49"/>
-    <mergeCell ref="A1:N1"/>
-    <mergeCell ref="G9:J9"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="A2:N2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="51" orientation="landscape"/>
@@ -5642,28 +5624,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="397"/>
-      <c r="C1" s="398"/>
-      <c r="D1" s="398"/>
-      <c r="E1" s="399"/>
-      <c r="F1" s="400"/>
-      <c r="G1" s="401"/>
-      <c r="H1" s="401"/>
-      <c r="I1" s="401"/>
-      <c r="J1" s="401"/>
-      <c r="K1" s="401"/>
-      <c r="L1" s="401"/>
-      <c r="M1" s="396"/>
-      <c r="N1" s="401"/>
-      <c r="O1" s="417"/>
-      <c r="P1" s="417"/>
-      <c r="Q1" s="417"/>
-      <c r="R1" s="396"/>
-      <c r="S1" s="417"/>
-      <c r="T1" s="396"/>
-      <c r="U1" s="401"/>
-      <c r="V1" s="417"/>
-      <c r="W1" s="401"/>
+      <c r="B1" s="407"/>
+      <c r="C1" s="408"/>
+      <c r="D1" s="408"/>
+      <c r="E1" s="409"/>
+      <c r="F1" s="401"/>
+      <c r="G1" s="392"/>
+      <c r="H1" s="392"/>
+      <c r="I1" s="392"/>
+      <c r="J1" s="392"/>
+      <c r="K1" s="392"/>
+      <c r="L1" s="392"/>
+      <c r="M1" s="402"/>
+      <c r="N1" s="392"/>
+      <c r="O1" s="415"/>
+      <c r="P1" s="415"/>
+      <c r="Q1" s="415"/>
+      <c r="R1" s="402"/>
+      <c r="S1" s="415"/>
+      <c r="T1" s="402"/>
+      <c r="U1" s="392"/>
+      <c r="V1" s="415"/>
+      <c r="W1" s="392"/>
     </row>
     <row r="2" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="113"/>
@@ -5733,7 +5715,7 @@
       <c r="R5" s="112"/>
       <c r="S5" s="112"/>
       <c r="T5" s="112" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="U5" s="4"/>
       <c r="V5" s="4"/>
@@ -5745,46 +5727,46 @@
         <v>7</v>
       </c>
       <c r="C6" s="271" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="D6" s="271" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="E6" s="272" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="F6" s="273" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="G6" s="276" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="H6" s="369" t="s">
         <v>61</v>
       </c>
       <c r="I6" s="276" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="J6" s="276" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="K6" s="274" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="L6" s="274" t="s">
         <v>39</v>
       </c>
       <c r="M6" s="274" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="N6" s="274" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="O6" s="274" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="P6" s="274" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="Q6" s="274" t="s">
         <v>168</v>
@@ -5796,7 +5778,7 @@
         <v>45</v>
       </c>
       <c r="T6" s="274" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="U6" s="274" t="s">
         <v>41</v>
@@ -8330,7 +8312,7 @@
     </row>
     <row r="108" spans="2:22" x14ac:dyDescent="0.3">
       <c r="E108" s="108" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="F108" s="88"/>
       <c r="G108" s="297">
@@ -8360,7 +8342,7 @@
     </row>
     <row r="111" spans="2:22" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="E111" s="109" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="G111" s="99">
         <f>SUM(G7:G107)</f>
@@ -8380,11 +8362,11 @@
       <c r="U112" s="3"/>
     </row>
     <row r="115" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E115" s="402" t="s">
+      <c r="E115" s="403" t="s">
         <v>55</v>
       </c>
-      <c r="F115" s="392"/>
-      <c r="G115" s="393"/>
+      <c r="F115" s="404"/>
+      <c r="G115" s="405"/>
       <c r="J115" s="127" t="s">
         <v>56</v>
       </c>
@@ -8513,10 +8495,10 @@
     </row>
     <row r="125" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E125" s="167" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="F125" s="161" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="G125" s="39" t="s">
         <v>32</v>
@@ -8525,10 +8507,10 @@
         <v>53</v>
       </c>
       <c r="I125" s="39" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="J125" s="39" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="K125" s="39" t="s">
         <v>15</v>
@@ -8828,31 +8810,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="397"/>
-      <c r="C1" s="413"/>
-      <c r="D1" s="396"/>
-      <c r="E1" s="400"/>
-      <c r="F1" s="414"/>
-      <c r="G1" s="414"/>
-      <c r="H1" s="414"/>
-      <c r="I1" s="415"/>
-      <c r="J1" s="396"/>
-      <c r="K1" s="396"/>
-      <c r="L1" s="396"/>
-      <c r="M1" s="396"/>
-      <c r="N1" s="396"/>
-      <c r="O1" s="396"/>
-      <c r="P1" s="417"/>
-      <c r="Q1" s="396"/>
-      <c r="R1" s="396"/>
-      <c r="S1" s="396"/>
-      <c r="T1" s="396"/>
-      <c r="U1" s="396"/>
-      <c r="V1" s="401"/>
-      <c r="W1" s="417"/>
-      <c r="X1" s="417"/>
-      <c r="Y1" s="401"/>
-      <c r="Z1" s="401"/>
+      <c r="B1" s="407"/>
+      <c r="C1" s="411"/>
+      <c r="D1" s="402"/>
+      <c r="E1" s="401"/>
+      <c r="F1" s="412"/>
+      <c r="G1" s="412"/>
+      <c r="H1" s="412"/>
+      <c r="I1" s="413"/>
+      <c r="J1" s="402"/>
+      <c r="K1" s="402"/>
+      <c r="L1" s="402"/>
+      <c r="M1" s="402"/>
+      <c r="N1" s="402"/>
+      <c r="O1" s="402"/>
+      <c r="P1" s="415"/>
+      <c r="Q1" s="402"/>
+      <c r="R1" s="402"/>
+      <c r="S1" s="402"/>
+      <c r="T1" s="402"/>
+      <c r="U1" s="402"/>
+      <c r="V1" s="392"/>
+      <c r="W1" s="415"/>
+      <c r="X1" s="415"/>
+      <c r="Y1" s="392"/>
+      <c r="Z1" s="392"/>
     </row>
     <row r="2" spans="2:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="113"/>
@@ -8931,22 +8913,22 @@
     </row>
     <row r="7" spans="2:27" x14ac:dyDescent="0.3">
       <c r="D7" s="208" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="E7" s="176" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="H7" s="209" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="I7" s="210" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="K7" s="208" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="L7" s="208" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
     </row>
     <row r="8" spans="2:27" s="7" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -8954,7 +8936,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="79" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>52</v>
@@ -8963,40 +8945,40 @@
         <v>11</v>
       </c>
       <c r="F8" s="48" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="G8" s="51" t="s">
         <v>61</v>
       </c>
       <c r="H8" s="48" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="I8" s="67" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="J8" s="12" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="K8" s="12" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="L8" s="12" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="M8" s="12" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="N8" s="12" t="s">
         <v>39</v>
       </c>
       <c r="O8" s="12" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="P8" s="12" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="Q8" s="12" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="R8" s="12" t="s">
         <v>168</v>
@@ -9008,7 +8990,7 @@
         <v>45</v>
       </c>
       <c r="U8" s="12" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="V8" s="12" t="s">
         <v>41</v>
@@ -9017,7 +8999,7 @@
         <v>46</v>
       </c>
       <c r="X8" s="12" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
     </row>
     <row r="9" spans="2:27" x14ac:dyDescent="0.3">
@@ -9811,17 +9793,17 @@
       <c r="M34" s="14"/>
     </row>
     <row r="37" spans="3:22" x14ac:dyDescent="0.3">
-      <c r="D37" s="402" t="s">
+      <c r="D37" s="403" t="s">
         <v>55</v>
       </c>
-      <c r="E37" s="392"/>
-      <c r="F37" s="393"/>
+      <c r="E37" s="404"/>
+      <c r="F37" s="405"/>
       <c r="G37" s="8"/>
-      <c r="J37" s="402" t="s">
+      <c r="J37" s="403" t="s">
         <v>56</v>
       </c>
-      <c r="K37" s="392"/>
-      <c r="L37" s="393"/>
+      <c r="K37" s="404"/>
+      <c r="L37" s="405"/>
     </row>
     <row r="38" spans="3:22" x14ac:dyDescent="0.3">
       <c r="D38" s="16" t="s">
@@ -9941,7 +9923,7 @@
     </row>
     <row r="48" spans="3:22" x14ac:dyDescent="0.3">
       <c r="G48" s="162" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="H48" s="162" t="s">
         <v>32</v>
@@ -9955,7 +9937,7 @@
     </row>
     <row r="49" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G49" s="46" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="H49" s="46">
         <f>SUMIF($J$9:$J$29,G49,$F$9:$F$29)</f>
@@ -9972,7 +9954,7 @@
     </row>
     <row r="50" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G50" s="46" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="H50" s="46">
         <f>SUMIF($J$9:$J$29,G50,$F$9:$F$29)</f>
@@ -9989,7 +9971,7 @@
     </row>
     <row r="51" spans="7:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G51" s="97" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="H51" s="97">
         <f>SUMIF($J$9:$J$29,G51,$F$9:$F$29)</f>
@@ -10133,31 +10115,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="397"/>
-      <c r="C1" s="413"/>
-      <c r="D1" s="396"/>
-      <c r="E1" s="400"/>
-      <c r="F1" s="414"/>
-      <c r="G1" s="414"/>
-      <c r="H1" s="414"/>
-      <c r="I1" s="415"/>
-      <c r="J1" s="396"/>
-      <c r="K1" s="396"/>
-      <c r="L1" s="396"/>
-      <c r="M1" s="396"/>
-      <c r="N1" s="396"/>
-      <c r="O1" s="396"/>
-      <c r="P1" s="417"/>
-      <c r="Q1" s="396"/>
-      <c r="R1" s="396"/>
-      <c r="S1" s="396"/>
-      <c r="T1" s="396"/>
-      <c r="U1" s="396"/>
-      <c r="V1" s="401"/>
-      <c r="W1" s="417"/>
-      <c r="X1" s="417"/>
-      <c r="Y1" s="401"/>
-      <c r="Z1" s="401"/>
+      <c r="B1" s="407"/>
+      <c r="C1" s="411"/>
+      <c r="D1" s="402"/>
+      <c r="E1" s="401"/>
+      <c r="F1" s="412"/>
+      <c r="G1" s="412"/>
+      <c r="H1" s="412"/>
+      <c r="I1" s="413"/>
+      <c r="J1" s="402"/>
+      <c r="K1" s="402"/>
+      <c r="L1" s="402"/>
+      <c r="M1" s="402"/>
+      <c r="N1" s="402"/>
+      <c r="O1" s="402"/>
+      <c r="P1" s="415"/>
+      <c r="Q1" s="402"/>
+      <c r="R1" s="402"/>
+      <c r="S1" s="402"/>
+      <c r="T1" s="402"/>
+      <c r="U1" s="402"/>
+      <c r="V1" s="392"/>
+      <c r="W1" s="415"/>
+      <c r="X1" s="415"/>
+      <c r="Y1" s="392"/>
+      <c r="Z1" s="392"/>
     </row>
     <row r="2" spans="2:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="113"/>
@@ -10236,22 +10218,22 @@
     </row>
     <row r="7" spans="2:27" x14ac:dyDescent="0.3">
       <c r="D7" s="208" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="E7" s="176" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="H7" s="209" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="I7" s="210" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="K7" s="208" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="L7" s="208" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
     </row>
     <row r="8" spans="2:27" s="7" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -10259,7 +10241,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="79" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>52</v>
@@ -10268,40 +10250,40 @@
         <v>11</v>
       </c>
       <c r="F8" s="48" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="G8" s="51" t="s">
         <v>61</v>
       </c>
       <c r="H8" s="48" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="I8" s="67" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="J8" s="12" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="K8" s="12" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="L8" s="12" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="M8" s="12" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="N8" s="12" t="s">
         <v>39</v>
       </c>
       <c r="O8" s="12" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="P8" s="12" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="Q8" s="12" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="R8" s="12" t="s">
         <v>168</v>
@@ -10313,7 +10295,7 @@
         <v>45</v>
       </c>
       <c r="U8" s="12" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="V8" s="12" t="s">
         <v>41</v>
@@ -10322,7 +10304,7 @@
         <v>46</v>
       </c>
       <c r="X8" s="12" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
     </row>
     <row r="9" spans="2:27" x14ac:dyDescent="0.3">
@@ -11116,17 +11098,17 @@
       <c r="M34" s="14"/>
     </row>
     <row r="37" spans="3:22" x14ac:dyDescent="0.3">
-      <c r="D37" s="402" t="s">
+      <c r="D37" s="403" t="s">
         <v>55</v>
       </c>
-      <c r="E37" s="392"/>
-      <c r="F37" s="393"/>
+      <c r="E37" s="404"/>
+      <c r="F37" s="405"/>
       <c r="G37" s="8"/>
-      <c r="J37" s="402" t="s">
+      <c r="J37" s="403" t="s">
         <v>56</v>
       </c>
-      <c r="K37" s="392"/>
-      <c r="L37" s="393"/>
+      <c r="K37" s="404"/>
+      <c r="L37" s="405"/>
     </row>
     <row r="38" spans="3:22" x14ac:dyDescent="0.3">
       <c r="D38" s="16" t="s">
@@ -11246,7 +11228,7 @@
     </row>
     <row r="48" spans="3:22" x14ac:dyDescent="0.3">
       <c r="G48" s="162" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="H48" s="162" t="s">
         <v>32</v>
@@ -11260,7 +11242,7 @@
     </row>
     <row r="49" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G49" s="46" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="H49" s="46">
         <f>SUMIF($J$9:$J$29,G49,$F$9:$F$29)</f>
@@ -11277,7 +11259,7 @@
     </row>
     <row r="50" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G50" s="46" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="H50" s="46">
         <f>SUMIF($J$9:$J$29,G50,$F$9:$F$29)</f>
@@ -11294,7 +11276,7 @@
     </row>
     <row r="51" spans="7:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G51" s="97" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="H51" s="97">
         <f>SUMIF($J$9:$J$29,G51,$F$9:$F$29)</f>
@@ -11421,42 +11403,42 @@
   <sheetData>
     <row r="1" spans="1:28" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="21" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="B1" s="21" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="G1" s="21" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="H1" s="21" t="s">
         <v>39</v>
       </c>
       <c r="I1" s="39" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="AB1" s="39" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="B2" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="C2" t="s">
         <v>59</v>
@@ -11468,94 +11450,94 @@
         <v>59</v>
       </c>
       <c r="F2" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="G2" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="H2" s="32" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="I2" s="8" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
       <c r="V2" s="8" t="s">
         <v>59</v>
       </c>
       <c r="AB2" s="8" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="B3" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="C3" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="D3" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="E3" t="s">
         <v>58</v>
       </c>
       <c r="F3" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="G3" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="H3">
         <f>Overview!C13</f>
         <v>0</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="V3" s="8" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="AB3" s="8" t="s">
-        <v>290</v>
+        <v>283</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="B4" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="C4" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="D4" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="E4" t="s">
         <v>57</v>
       </c>
       <c r="F4" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="G4" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="H4" s="32">
         <f>Overview!C16</f>
         <v>0</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="V4" s="8" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="AB4" s="8" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.3">
@@ -11563,13 +11545,13 @@
         <v>93</v>
       </c>
       <c r="D5" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="F5" t="s">
         <v>103</v>
       </c>
       <c r="G5" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="H5" s="32">
         <f>Overview!C17</f>
@@ -11579,51 +11561,51 @@
         <v>0</v>
       </c>
       <c r="V5" s="8" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="AB5" s="8" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="H6" s="32">
         <f>Overview!C18</f>
         <v>0</v>
       </c>
       <c r="AB6" s="8" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="H7" s="32">
         <f>Overview!C19</f>
         <v>0</v>
       </c>
       <c r="AB7" s="8" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="H8" s="32">
         <f>Overview!C20</f>
         <v>0</v>
       </c>
       <c r="AB8" s="8" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="H9" s="32">
         <f>Overview!C21</f>
@@ -11781,14 +11763,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:12" ht="33.75" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="C2" s="411" t="s">
+      <c r="C2" s="391" t="s">
         <v>162</v>
       </c>
-      <c r="D2" s="401"/>
-      <c r="E2" s="401"/>
-      <c r="F2" s="401"/>
-      <c r="G2" s="401"/>
-      <c r="H2" s="401"/>
+      <c r="D2" s="392"/>
+      <c r="E2" s="392"/>
+      <c r="F2" s="392"/>
+      <c r="G2" s="392"/>
+      <c r="H2" s="392"/>
       <c r="I2" s="217"/>
     </row>
     <row r="3" spans="1:12" ht="33.75" customHeight="1" x14ac:dyDescent="0.65">
@@ -11973,7 +11955,7 @@
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="B2:K94"/>
+  <dimension ref="B2:L94"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="5.109375" style="8" customWidth="1"/>
@@ -11982,28 +11964,28 @@
     <col min="5" max="5" width="29" customWidth="1"/>
     <col min="6" max="6" width="14.44140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="23.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="41.33203125" customWidth="1"/>
-    <col min="9" max="9" width="5.109375" customWidth="1"/>
-    <col min="10" max="10" width="30.33203125" customWidth="1"/>
-    <col min="11" max="11" width="21.33203125" customWidth="1"/>
+    <col min="8" max="9" width="41.33203125" customWidth="1"/>
+    <col min="10" max="10" width="5.109375" customWidth="1"/>
+    <col min="11" max="11" width="30.33203125" customWidth="1"/>
+    <col min="12" max="12" width="21.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" ht="33.75" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="C2" s="411" t="s">
+    <row r="2" spans="2:12" ht="33.75" customHeight="1" x14ac:dyDescent="0.65">
+      <c r="C2" s="391" t="s">
         <v>191</v>
       </c>
-      <c r="D2" s="401"/>
-      <c r="E2" s="401"/>
-      <c r="F2" s="401"/>
-      <c r="G2" s="401"/>
-      <c r="H2" s="401"/>
-    </row>
-    <row r="3" spans="2:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D2" s="392"/>
+      <c r="E2" s="392"/>
+      <c r="F2" s="392"/>
+      <c r="G2" s="392"/>
+      <c r="H2" s="392"/>
+    </row>
+    <row r="3" spans="2:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D3" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
       <c r="C4" s="274" t="s">
         <v>193</v>
       </c>
@@ -12022,55 +12004,50 @@
       <c r="H4" s="276" t="s">
         <v>198</v>
       </c>
-      <c r="J4" s="331" t="s">
+      <c r="I4" s="276" t="s">
+        <v>303</v>
+      </c>
+      <c r="K4" s="331" t="s">
         <v>199</v>
       </c>
-      <c r="K4" s="332">
+      <c r="L4" s="332">
         <f>Overview!C9</f>
         <v>46068</v>
       </c>
     </row>
-    <row r="5" spans="2:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B5" s="8">
         <v>1</v>
       </c>
-      <c r="C5" s="221" t="s">
-        <v>200</v>
-      </c>
+      <c r="C5" s="221"/>
       <c r="D5" s="221"/>
       <c r="E5" s="117"/>
-      <c r="F5" s="104" t="s">
-        <v>201</v>
-      </c>
+      <c r="F5" s="104"/>
       <c r="G5" s="104"/>
       <c r="H5" s="36"/>
-      <c r="J5" s="333" t="s">
-        <v>202</v>
-      </c>
-      <c r="K5" s="334">
-        <f>K4-120</f>
+      <c r="I5" s="36"/>
+      <c r="K5" s="333" t="s">
+        <v>200</v>
+      </c>
+      <c r="L5" s="334">
+        <f>L4-120</f>
         <v>45948</v>
       </c>
     </row>
-    <row r="6" spans="2:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="8">
-        <f t="shared" ref="B6:B53" si="0">B5+1</f>
         <v>2</v>
       </c>
-      <c r="C6" s="221" t="s">
-        <v>203</v>
-      </c>
+      <c r="C6" s="221"/>
       <c r="D6" s="221"/>
       <c r="E6" s="117"/>
-      <c r="F6" s="104" t="s">
-        <v>201</v>
-      </c>
+      <c r="F6" s="104"/>
       <c r="G6" s="104"/>
       <c r="H6" s="36"/>
-    </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="I6" s="36"/>
+    </row>
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B7" s="8">
-        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="C7" s="221"/>
@@ -12079,17 +12056,17 @@
       <c r="F7" s="104"/>
       <c r="G7" s="104"/>
       <c r="H7" s="36"/>
-      <c r="J7" s="335" t="s">
-        <v>204</v>
-      </c>
-      <c r="K7" s="336">
+      <c r="I7" s="36"/>
+      <c r="K7" s="335" t="s">
+        <v>201</v>
+      </c>
+      <c r="L7" s="336">
         <f>COUNTIF(F5:F89,"Y")</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="8">
-        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C8" s="221"/>
@@ -12098,17 +12075,17 @@
       <c r="F8" s="104"/>
       <c r="G8" s="104"/>
       <c r="H8" s="36"/>
-      <c r="J8" s="337" t="s">
-        <v>205</v>
-      </c>
-      <c r="K8" s="338">
+      <c r="I8" s="36"/>
+      <c r="K8" s="337" t="s">
+        <v>202</v>
+      </c>
+      <c r="L8" s="338">
         <f>COUNTA(C5:C90)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="2:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="8">
-        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C9" s="159"/>
@@ -12117,17 +12094,17 @@
       <c r="F9" s="104"/>
       <c r="G9" s="104"/>
       <c r="H9" s="36"/>
-      <c r="J9" s="339" t="s">
+      <c r="I9" s="36"/>
+      <c r="K9" s="339" t="s">
         <v>146</v>
       </c>
-      <c r="K9" s="340">
-        <f>K7/K8</f>
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="L9" s="340" t="e">
+        <f>L7/L8</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B10" s="8">
-        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C10" s="221"/>
@@ -12136,10 +12113,10 @@
       <c r="F10" s="104"/>
       <c r="G10" s="104"/>
       <c r="H10" s="36"/>
-    </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="I10" s="36"/>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="8">
-        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C11" s="221"/>
@@ -12148,10 +12125,10 @@
       <c r="F11" s="104"/>
       <c r="G11" s="104"/>
       <c r="H11" s="36"/>
-    </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="I11" s="36"/>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="8">
-        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C12" s="221"/>
@@ -12160,10 +12137,10 @@
       <c r="F12" s="104"/>
       <c r="G12" s="104"/>
       <c r="H12" s="36"/>
-    </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="I12" s="36"/>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="8">
-        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C13" s="159"/>
@@ -12172,10 +12149,10 @@
       <c r="F13" s="104"/>
       <c r="G13" s="104"/>
       <c r="H13" s="36"/>
-    </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="I13" s="36"/>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="8">
-        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C14" s="221"/>
@@ -12184,10 +12161,10 @@
       <c r="F14" s="104"/>
       <c r="G14" s="104"/>
       <c r="H14" s="36"/>
-    </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="I14" s="36"/>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="8">
-        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C15" s="221"/>
@@ -12196,10 +12173,10 @@
       <c r="F15" s="104"/>
       <c r="G15" s="104"/>
       <c r="H15" s="36"/>
-    </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="I15" s="36"/>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="8">
-        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C16" s="221"/>
@@ -12208,10 +12185,10 @@
       <c r="F16" s="104"/>
       <c r="G16" s="104"/>
       <c r="H16" s="36"/>
-    </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I16" s="36"/>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B17" s="8">
-        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C17" s="221"/>
@@ -12220,10 +12197,10 @@
       <c r="F17" s="104"/>
       <c r="G17" s="104"/>
       <c r="H17" s="36"/>
-    </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I17" s="36"/>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B18" s="8">
-        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C18" s="159"/>
@@ -12232,10 +12209,10 @@
       <c r="F18" s="104"/>
       <c r="G18" s="104"/>
       <c r="H18" s="36"/>
-    </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I18" s="36"/>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B19" s="8">
-        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="C19" s="221"/>
@@ -12244,10 +12221,10 @@
       <c r="F19" s="104"/>
       <c r="G19" s="104"/>
       <c r="H19" s="36"/>
-    </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I19" s="36"/>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B20" s="8">
-        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="C20" s="159"/>
@@ -12256,10 +12233,10 @@
       <c r="F20" s="104"/>
       <c r="G20" s="104"/>
       <c r="H20" s="36"/>
-    </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I20" s="36"/>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B21" s="8">
-        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="C21" s="159"/>
@@ -12268,10 +12245,10 @@
       <c r="F21" s="104"/>
       <c r="G21" s="104"/>
       <c r="H21" s="36"/>
-    </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I21" s="36"/>
+    </row>
+    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B22" s="8">
-        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C22" s="221"/>
@@ -12280,10 +12257,10 @@
       <c r="F22" s="104"/>
       <c r="G22" s="104"/>
       <c r="H22" s="36"/>
-    </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I22" s="36"/>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B23" s="8">
-        <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="C23" s="221"/>
@@ -12292,10 +12269,10 @@
       <c r="F23" s="104"/>
       <c r="G23" s="104"/>
       <c r="H23" s="36"/>
-    </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I23" s="36"/>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B24" s="8">
-        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="C24" s="159"/>
@@ -12304,10 +12281,10 @@
       <c r="F24" s="104"/>
       <c r="G24" s="104"/>
       <c r="H24" s="36"/>
-    </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I24" s="36"/>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B25" s="8">
-        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="C25" s="159"/>
@@ -12316,10 +12293,10 @@
       <c r="F25" s="104"/>
       <c r="G25" s="104"/>
       <c r="H25" s="36"/>
-    </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I25" s="36"/>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B26" s="8">
-        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="C26" s="159"/>
@@ -12328,10 +12305,10 @@
       <c r="F26" s="104"/>
       <c r="G26" s="104"/>
       <c r="H26" s="36"/>
-    </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I26" s="36"/>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B27" s="8">
-        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="C27" s="159"/>
@@ -12340,10 +12317,10 @@
       <c r="F27" s="104"/>
       <c r="G27" s="104"/>
       <c r="H27" s="36"/>
-    </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I27" s="36"/>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B28" s="8">
-        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C28" s="159"/>
@@ -12352,10 +12329,10 @@
       <c r="F28" s="104"/>
       <c r="G28" s="104"/>
       <c r="H28" s="36"/>
-    </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I28" s="36"/>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B29" s="8">
-        <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="C29" s="221"/>
@@ -12364,10 +12341,10 @@
       <c r="F29" s="104"/>
       <c r="G29" s="104"/>
       <c r="H29" s="36"/>
-    </row>
-    <row r="30" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I29" s="36"/>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B30" s="8">
-        <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="C30" s="221"/>
@@ -12376,10 +12353,10 @@
       <c r="F30" s="104"/>
       <c r="G30" s="104"/>
       <c r="H30" s="36"/>
-    </row>
-    <row r="31" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I30" s="36"/>
+    </row>
+    <row r="31" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B31" s="8">
-        <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="C31" s="159"/>
@@ -12388,10 +12365,10 @@
       <c r="F31" s="104"/>
       <c r="G31" s="104"/>
       <c r="H31" s="36"/>
-    </row>
-    <row r="32" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I31" s="36"/>
+    </row>
+    <row r="32" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B32" s="8">
-        <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="C32" s="221"/>
@@ -12400,10 +12377,10 @@
       <c r="F32" s="104"/>
       <c r="G32" s="104"/>
       <c r="H32" s="36"/>
-    </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I32" s="36"/>
+    </row>
+    <row r="33" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B33" s="8">
-        <f t="shared" si="0"/>
         <v>29</v>
       </c>
       <c r="C33" s="221"/>
@@ -12412,10 +12389,10 @@
       <c r="F33" s="104"/>
       <c r="G33" s="104"/>
       <c r="H33" s="36"/>
-    </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I33" s="36"/>
+    </row>
+    <row r="34" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B34" s="8">
-        <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C34" s="221"/>
@@ -12424,10 +12401,10 @@
       <c r="F34" s="104"/>
       <c r="G34" s="104"/>
       <c r="H34" s="36"/>
-    </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I34" s="36"/>
+    </row>
+    <row r="35" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B35" s="8">
-        <f t="shared" si="0"/>
         <v>31</v>
       </c>
       <c r="C35" s="221"/>
@@ -12436,10 +12413,10 @@
       <c r="F35" s="104"/>
       <c r="G35" s="104"/>
       <c r="H35" s="36"/>
-    </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I35" s="36"/>
+    </row>
+    <row r="36" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B36" s="8">
-        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C36" s="221"/>
@@ -12448,10 +12425,10 @@
       <c r="F36" s="104"/>
       <c r="G36" s="104"/>
       <c r="H36" s="36"/>
-    </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I36" s="36"/>
+    </row>
+    <row r="37" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B37" s="8">
-        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="C37" s="221"/>
@@ -12460,10 +12437,10 @@
       <c r="F37" s="104"/>
       <c r="G37" s="104"/>
       <c r="H37" s="36"/>
-    </row>
-    <row r="38" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I37" s="36"/>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B38" s="8">
-        <f t="shared" si="0"/>
         <v>34</v>
       </c>
       <c r="C38" s="221"/>
@@ -12472,10 +12449,10 @@
       <c r="F38" s="104"/>
       <c r="G38" s="104"/>
       <c r="H38" s="36"/>
-    </row>
-    <row r="39" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I38" s="36"/>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B39" s="8">
-        <f t="shared" si="0"/>
         <v>35</v>
       </c>
       <c r="C39" s="221"/>
@@ -12484,10 +12461,10 @@
       <c r="F39" s="104"/>
       <c r="G39" s="104"/>
       <c r="H39" s="36"/>
-    </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I39" s="36"/>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B40" s="8">
-        <f t="shared" si="0"/>
         <v>36</v>
       </c>
       <c r="C40" s="221"/>
@@ -12496,10 +12473,10 @@
       <c r="F40" s="104"/>
       <c r="G40" s="104"/>
       <c r="H40" s="36"/>
-    </row>
-    <row r="41" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I40" s="36"/>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B41" s="8">
-        <f t="shared" si="0"/>
         <v>37</v>
       </c>
       <c r="C41" s="221"/>
@@ -12508,10 +12485,10 @@
       <c r="F41" s="104"/>
       <c r="G41" s="104"/>
       <c r="H41" s="36"/>
-    </row>
-    <row r="42" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I41" s="36"/>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B42" s="8">
-        <f t="shared" si="0"/>
         <v>38</v>
       </c>
       <c r="C42" s="221"/>
@@ -12520,10 +12497,10 @@
       <c r="F42" s="104"/>
       <c r="G42" s="104"/>
       <c r="H42" s="36"/>
-    </row>
-    <row r="43" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I42" s="36"/>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B43" s="8">
-        <f t="shared" si="0"/>
         <v>39</v>
       </c>
       <c r="C43" s="221"/>
@@ -12532,10 +12509,10 @@
       <c r="F43" s="104"/>
       <c r="G43" s="104"/>
       <c r="H43" s="36"/>
-    </row>
-    <row r="44" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I43" s="36"/>
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B44" s="8">
-        <f t="shared" si="0"/>
         <v>40</v>
       </c>
       <c r="C44" s="159"/>
@@ -12544,10 +12521,10 @@
       <c r="F44" s="104"/>
       <c r="G44" s="104"/>
       <c r="H44" s="36"/>
-    </row>
-    <row r="45" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I44" s="36"/>
+    </row>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B45" s="8">
-        <f t="shared" si="0"/>
         <v>41</v>
       </c>
       <c r="C45" s="159"/>
@@ -12556,10 +12533,10 @@
       <c r="F45" s="104"/>
       <c r="G45" s="104"/>
       <c r="H45" s="36"/>
-    </row>
-    <row r="46" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I45" s="36"/>
+    </row>
+    <row r="46" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B46" s="8">
-        <f t="shared" si="0"/>
         <v>42</v>
       </c>
       <c r="C46" s="159"/>
@@ -12568,10 +12545,10 @@
       <c r="F46" s="104"/>
       <c r="G46" s="104"/>
       <c r="H46" s="36"/>
-    </row>
-    <row r="47" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I46" s="36"/>
+    </row>
+    <row r="47" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B47" s="8">
-        <f t="shared" si="0"/>
         <v>43</v>
       </c>
       <c r="C47" s="221"/>
@@ -12580,10 +12557,10 @@
       <c r="F47" s="104"/>
       <c r="G47" s="104"/>
       <c r="H47" s="36"/>
-    </row>
-    <row r="48" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I47" s="36"/>
+    </row>
+    <row r="48" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B48" s="8">
-        <f t="shared" si="0"/>
         <v>44</v>
       </c>
       <c r="C48" s="159"/>
@@ -12592,10 +12569,10 @@
       <c r="F48" s="104"/>
       <c r="G48" s="104"/>
       <c r="H48" s="36"/>
-    </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I48" s="36"/>
+    </row>
+    <row r="49" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B49" s="8">
-        <f t="shared" si="0"/>
         <v>45</v>
       </c>
       <c r="C49" s="221"/>
@@ -12604,10 +12581,10 @@
       <c r="F49" s="104"/>
       <c r="G49" s="104"/>
       <c r="H49" s="36"/>
-    </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I49" s="36"/>
+    </row>
+    <row r="50" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B50" s="8">
-        <f t="shared" si="0"/>
         <v>46</v>
       </c>
       <c r="C50" s="221"/>
@@ -12616,10 +12593,10 @@
       <c r="F50" s="104"/>
       <c r="G50" s="104"/>
       <c r="H50" s="36"/>
-    </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I50" s="36"/>
+    </row>
+    <row r="51" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B51" s="8">
-        <f t="shared" si="0"/>
         <v>47</v>
       </c>
       <c r="C51" s="221"/>
@@ -12628,10 +12605,10 @@
       <c r="F51" s="104"/>
       <c r="G51" s="104"/>
       <c r="H51" s="36"/>
-    </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I51" s="36"/>
+    </row>
+    <row r="52" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B52" s="8">
-        <f t="shared" si="0"/>
         <v>48</v>
       </c>
       <c r="C52" s="159"/>
@@ -12640,10 +12617,10 @@
       <c r="F52" s="104"/>
       <c r="G52" s="104"/>
       <c r="H52" s="36"/>
-    </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I52" s="36"/>
+    </row>
+    <row r="53" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B53" s="8">
-        <f t="shared" si="0"/>
         <v>49</v>
       </c>
       <c r="C53" s="221"/>
@@ -12652,58 +12629,47 @@
       <c r="F53" s="104"/>
       <c r="G53" s="104"/>
       <c r="H53" s="36"/>
-    </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I53" s="36"/>
+    </row>
+    <row r="54" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B54" s="8">
-        <v>1</v>
-      </c>
-      <c r="C54" s="221" t="s">
-        <v>206</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="C54" s="221"/>
       <c r="D54" s="221"/>
       <c r="E54" s="117"/>
-      <c r="F54" s="104" t="s">
-        <v>201</v>
-      </c>
+      <c r="F54" s="104"/>
       <c r="G54" s="104"/>
       <c r="H54" s="36"/>
-    </row>
-    <row r="55" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I54" s="36"/>
+    </row>
+    <row r="55" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B55" s="8">
-        <f t="shared" ref="B55:B79" si="1">B54+1</f>
-        <v>2</v>
-      </c>
-      <c r="C55" s="221" t="s">
-        <v>207</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="C55" s="221"/>
       <c r="D55" s="221"/>
       <c r="E55" s="117"/>
-      <c r="F55" s="104" t="s">
-        <v>201</v>
-      </c>
+      <c r="F55" s="104"/>
       <c r="G55" s="104"/>
       <c r="H55" s="36"/>
-    </row>
-    <row r="56" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I55" s="36"/>
+    </row>
+    <row r="56" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B56" s="8">
-        <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="C56" s="159" t="s">
-        <v>208</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="C56" s="159"/>
       <c r="D56" s="159"/>
       <c r="E56" s="117"/>
-      <c r="F56" s="104" t="s">
-        <v>209</v>
-      </c>
+      <c r="F56" s="104"/>
       <c r="G56" s="104"/>
       <c r="H56" s="36"/>
-    </row>
-    <row r="57" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I56" s="36"/>
+    </row>
+    <row r="57" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B57" s="8">
-        <f t="shared" si="1"/>
-        <v>4</v>
+        <v>53</v>
       </c>
       <c r="C57" s="221"/>
       <c r="D57" s="221"/>
@@ -12711,11 +12677,11 @@
       <c r="F57" s="104"/>
       <c r="G57" s="104"/>
       <c r="H57" s="36"/>
-    </row>
-    <row r="58" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I57" s="36"/>
+    </row>
+    <row r="58" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B58" s="8">
-        <f t="shared" si="1"/>
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="C58" s="221"/>
       <c r="D58" s="221"/>
@@ -12723,11 +12689,11 @@
       <c r="F58" s="104"/>
       <c r="G58" s="104"/>
       <c r="H58" s="36"/>
-    </row>
-    <row r="59" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I58" s="36"/>
+    </row>
+    <row r="59" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B59" s="8">
-        <f t="shared" si="1"/>
-        <v>6</v>
+        <v>55</v>
       </c>
       <c r="C59" s="159"/>
       <c r="D59" s="159"/>
@@ -12735,11 +12701,11 @@
       <c r="F59" s="104"/>
       <c r="G59" s="104"/>
       <c r="H59" s="36"/>
-    </row>
-    <row r="60" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I59" s="36"/>
+    </row>
+    <row r="60" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B60" s="8">
-        <f t="shared" si="1"/>
-        <v>7</v>
+        <v>56</v>
       </c>
       <c r="C60" s="159"/>
       <c r="D60" s="159"/>
@@ -12747,11 +12713,11 @@
       <c r="F60" s="104"/>
       <c r="G60" s="104"/>
       <c r="H60" s="36"/>
-    </row>
-    <row r="61" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I60" s="36"/>
+    </row>
+    <row r="61" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B61" s="8">
-        <f t="shared" si="1"/>
-        <v>8</v>
+        <v>57</v>
       </c>
       <c r="C61" s="221"/>
       <c r="D61" s="221"/>
@@ -12759,11 +12725,11 @@
       <c r="F61" s="104"/>
       <c r="G61" s="104"/>
       <c r="H61" s="36"/>
-    </row>
-    <row r="62" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I61" s="36"/>
+    </row>
+    <row r="62" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B62" s="8">
-        <f t="shared" si="1"/>
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="C62" s="221"/>
       <c r="D62" s="221"/>
@@ -12771,11 +12737,11 @@
       <c r="F62" s="104"/>
       <c r="G62" s="104"/>
       <c r="H62" s="36"/>
-    </row>
-    <row r="63" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I62" s="36"/>
+    </row>
+    <row r="63" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B63" s="8">
-        <f t="shared" si="1"/>
-        <v>10</v>
+        <v>59</v>
       </c>
       <c r="C63" s="221"/>
       <c r="D63" s="221"/>
@@ -12783,11 +12749,11 @@
       <c r="F63" s="104"/>
       <c r="G63" s="104"/>
       <c r="H63" s="36"/>
-    </row>
-    <row r="64" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I63" s="36"/>
+    </row>
+    <row r="64" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B64" s="8">
-        <f t="shared" si="1"/>
-        <v>11</v>
+        <v>60</v>
       </c>
       <c r="C64" s="221"/>
       <c r="D64" s="221"/>
@@ -12795,11 +12761,11 @@
       <c r="F64" s="104"/>
       <c r="G64" s="104"/>
       <c r="H64" s="36"/>
-    </row>
-    <row r="65" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I64" s="36"/>
+    </row>
+    <row r="65" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B65" s="8">
-        <f t="shared" si="1"/>
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="C65" s="221"/>
       <c r="D65" s="221"/>
@@ -12807,11 +12773,11 @@
       <c r="F65" s="104"/>
       <c r="G65" s="104"/>
       <c r="H65" s="36"/>
-    </row>
-    <row r="66" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I65" s="36"/>
+    </row>
+    <row r="66" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B66" s="8">
-        <f t="shared" si="1"/>
-        <v>13</v>
+        <v>62</v>
       </c>
       <c r="C66" s="221"/>
       <c r="D66" s="221"/>
@@ -12819,11 +12785,11 @@
       <c r="F66" s="104"/>
       <c r="G66" s="104"/>
       <c r="H66" s="36"/>
-    </row>
-    <row r="67" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I66" s="36"/>
+    </row>
+    <row r="67" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B67" s="8">
-        <f t="shared" si="1"/>
-        <v>14</v>
+        <v>63</v>
       </c>
       <c r="C67" s="221"/>
       <c r="D67" s="221"/>
@@ -12831,11 +12797,11 @@
       <c r="F67" s="104"/>
       <c r="G67" s="104"/>
       <c r="H67" s="36"/>
-    </row>
-    <row r="68" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I67" s="36"/>
+    </row>
+    <row r="68" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B68" s="8">
-        <f t="shared" si="1"/>
-        <v>15</v>
+        <v>64</v>
       </c>
       <c r="C68" s="221"/>
       <c r="D68" s="221"/>
@@ -12843,11 +12809,11 @@
       <c r="F68" s="104"/>
       <c r="G68" s="104"/>
       <c r="H68" s="36"/>
-    </row>
-    <row r="69" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I68" s="36"/>
+    </row>
+    <row r="69" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B69" s="8">
-        <f t="shared" si="1"/>
-        <v>16</v>
+        <v>65</v>
       </c>
       <c r="C69" s="221"/>
       <c r="D69" s="221"/>
@@ -12855,11 +12821,11 @@
       <c r="F69" s="104"/>
       <c r="G69" s="104"/>
       <c r="H69" s="36"/>
-    </row>
-    <row r="70" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I69" s="36"/>
+    </row>
+    <row r="70" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B70" s="8">
-        <f t="shared" si="1"/>
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="C70" s="221"/>
       <c r="D70" s="221"/>
@@ -12867,11 +12833,11 @@
       <c r="F70" s="104"/>
       <c r="G70" s="104"/>
       <c r="H70" s="36"/>
-    </row>
-    <row r="71" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I70" s="36"/>
+    </row>
+    <row r="71" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B71" s="8">
-        <f t="shared" si="1"/>
-        <v>18</v>
+        <v>67</v>
       </c>
       <c r="C71" s="221"/>
       <c r="D71" s="221"/>
@@ -12879,11 +12845,11 @@
       <c r="F71" s="104"/>
       <c r="G71" s="104"/>
       <c r="H71" s="36"/>
-    </row>
-    <row r="72" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I71" s="36"/>
+    </row>
+    <row r="72" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B72" s="8">
-        <f t="shared" si="1"/>
-        <v>19</v>
+        <v>68</v>
       </c>
       <c r="C72" s="221"/>
       <c r="D72" s="221"/>
@@ -12891,11 +12857,11 @@
       <c r="F72" s="104"/>
       <c r="G72" s="104"/>
       <c r="H72" s="36"/>
-    </row>
-    <row r="73" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I72" s="36"/>
+    </row>
+    <row r="73" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B73" s="8">
-        <f t="shared" si="1"/>
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="C73" s="221"/>
       <c r="D73" s="221"/>
@@ -12903,11 +12869,11 @@
       <c r="F73" s="104"/>
       <c r="G73" s="104"/>
       <c r="H73" s="36"/>
-    </row>
-    <row r="74" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I73" s="36"/>
+    </row>
+    <row r="74" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B74" s="8">
-        <f t="shared" si="1"/>
-        <v>21</v>
+        <v>70</v>
       </c>
       <c r="C74" s="221"/>
       <c r="D74" s="221"/>
@@ -12915,11 +12881,11 @@
       <c r="F74" s="104"/>
       <c r="G74" s="104"/>
       <c r="H74" s="36"/>
-    </row>
-    <row r="75" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I74" s="36"/>
+    </row>
+    <row r="75" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B75" s="8">
-        <f t="shared" si="1"/>
-        <v>22</v>
+        <v>71</v>
       </c>
       <c r="C75" s="221"/>
       <c r="D75" s="221"/>
@@ -12927,11 +12893,11 @@
       <c r="F75" s="104"/>
       <c r="G75" s="104"/>
       <c r="H75" s="36"/>
-    </row>
-    <row r="76" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I75" s="36"/>
+    </row>
+    <row r="76" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B76" s="8">
-        <f t="shared" si="1"/>
-        <v>23</v>
+        <v>72</v>
       </c>
       <c r="C76" s="221"/>
       <c r="D76" s="221"/>
@@ -12939,11 +12905,11 @@
       <c r="F76" s="104"/>
       <c r="G76" s="104"/>
       <c r="H76" s="36"/>
-    </row>
-    <row r="77" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I76" s="36"/>
+    </row>
+    <row r="77" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B77" s="8">
-        <f t="shared" si="1"/>
-        <v>24</v>
+        <v>73</v>
       </c>
       <c r="C77" s="221"/>
       <c r="D77" s="221"/>
@@ -12951,11 +12917,11 @@
       <c r="F77" s="104"/>
       <c r="G77" s="104"/>
       <c r="H77" s="36"/>
-    </row>
-    <row r="78" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I77" s="36"/>
+    </row>
+    <row r="78" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B78" s="8">
-        <f t="shared" si="1"/>
-        <v>25</v>
+        <v>74</v>
       </c>
       <c r="C78" s="221"/>
       <c r="D78" s="221"/>
@@ -12963,11 +12929,11 @@
       <c r="F78" s="104"/>
       <c r="G78" s="104"/>
       <c r="H78" s="36"/>
-    </row>
-    <row r="79" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I78" s="36"/>
+    </row>
+    <row r="79" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B79" s="8">
-        <f t="shared" si="1"/>
-        <v>26</v>
+        <v>75</v>
       </c>
       <c r="C79" s="221"/>
       <c r="D79" s="221"/>
@@ -12975,10 +12941,11 @@
       <c r="F79" s="104"/>
       <c r="G79" s="104"/>
       <c r="H79" s="36"/>
-    </row>
-    <row r="80" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I79" s="36"/>
+    </row>
+    <row r="80" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B80" s="8">
-        <v>27</v>
+        <v>76</v>
       </c>
       <c r="C80" s="221"/>
       <c r="D80" s="221"/>
@@ -12986,10 +12953,11 @@
       <c r="F80" s="104"/>
       <c r="G80" s="104"/>
       <c r="H80" s="36"/>
-    </row>
-    <row r="81" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I80" s="36"/>
+    </row>
+    <row r="81" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B81" s="8">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="C81" s="221"/>
       <c r="D81" s="221"/>
@@ -12997,10 +12965,11 @@
       <c r="F81" s="104"/>
       <c r="G81" s="104"/>
       <c r="H81" s="36"/>
-    </row>
-    <row r="82" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I81" s="36"/>
+    </row>
+    <row r="82" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B82" s="8">
-        <v>29</v>
+        <v>78</v>
       </c>
       <c r="C82" s="221"/>
       <c r="D82" s="221"/>
@@ -13008,10 +12977,11 @@
       <c r="F82" s="104"/>
       <c r="G82" s="104"/>
       <c r="H82" s="36"/>
-    </row>
-    <row r="83" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I82" s="36"/>
+    </row>
+    <row r="83" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B83" s="8">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="C83" s="221"/>
       <c r="D83" s="221"/>
@@ -13019,10 +12989,11 @@
       <c r="F83" s="104"/>
       <c r="G83" s="104"/>
       <c r="H83" s="36"/>
-    </row>
-    <row r="84" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I83" s="36"/>
+    </row>
+    <row r="84" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B84" s="8">
-        <v>31</v>
+        <v>80</v>
       </c>
       <c r="C84" s="221"/>
       <c r="D84" s="221"/>
@@ -13030,10 +13001,11 @@
       <c r="F84" s="104"/>
       <c r="G84" s="104"/>
       <c r="H84" s="36"/>
-    </row>
-    <row r="85" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I84" s="36"/>
+    </row>
+    <row r="85" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B85" s="8">
-        <v>32</v>
+        <v>81</v>
       </c>
       <c r="C85" s="221"/>
       <c r="D85" s="221"/>
@@ -13041,10 +13013,11 @@
       <c r="F85" s="104"/>
       <c r="G85" s="104"/>
       <c r="H85" s="36"/>
-    </row>
-    <row r="86" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I85" s="36"/>
+    </row>
+    <row r="86" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B86" s="8">
-        <v>33</v>
+        <v>82</v>
       </c>
       <c r="C86" s="221"/>
       <c r="D86" s="221"/>
@@ -13052,10 +13025,11 @@
       <c r="F86" s="104"/>
       <c r="G86" s="104"/>
       <c r="H86" s="36"/>
-    </row>
-    <row r="87" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I86" s="36"/>
+    </row>
+    <row r="87" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B87" s="8">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="C87" s="221"/>
       <c r="D87" s="221"/>
@@ -13063,10 +13037,11 @@
       <c r="F87" s="104"/>
       <c r="G87" s="104"/>
       <c r="H87" s="36"/>
-    </row>
-    <row r="88" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I87" s="36"/>
+    </row>
+    <row r="88" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B88" s="8">
-        <v>35</v>
+        <v>84</v>
       </c>
       <c r="C88" s="221"/>
       <c r="D88" s="221"/>
@@ -13074,10 +13049,11 @@
       <c r="F88" s="104"/>
       <c r="G88" s="104"/>
       <c r="H88" s="36"/>
-    </row>
-    <row r="89" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I88" s="36"/>
+    </row>
+    <row r="89" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B89" s="8">
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="C89" s="221"/>
       <c r="D89" s="221"/>
@@ -13085,8 +13061,9 @@
       <c r="F89" s="104"/>
       <c r="G89" s="104"/>
       <c r="H89" s="36"/>
-    </row>
-    <row r="94" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I89" s="36"/>
+    </row>
+    <row r="94" spans="2:9" x14ac:dyDescent="0.3">
       <c r="F94" s="299"/>
       <c r="G94" s="299"/>
     </row>
@@ -13160,46 +13137,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:53" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="397"/>
-      <c r="C1" s="398"/>
-      <c r="D1" s="398"/>
-      <c r="E1" s="399"/>
-      <c r="F1" s="399"/>
-      <c r="G1" s="399"/>
-      <c r="H1" s="400"/>
-      <c r="I1" s="400"/>
-      <c r="J1" s="400"/>
-      <c r="K1" s="396"/>
-      <c r="L1" s="400"/>
-      <c r="M1" s="400"/>
-      <c r="N1" s="395"/>
-      <c r="O1" s="395"/>
-      <c r="P1" s="395"/>
-      <c r="Q1" s="395"/>
-      <c r="R1" s="395"/>
-      <c r="S1" s="395"/>
-      <c r="T1" s="395"/>
-      <c r="U1" s="395"/>
-      <c r="V1" s="395"/>
-      <c r="W1" s="395"/>
-      <c r="X1" s="395"/>
-      <c r="Y1" s="395"/>
-      <c r="Z1" s="395"/>
-      <c r="AA1" s="395"/>
-      <c r="AB1" s="395"/>
-      <c r="AC1" s="395"/>
-      <c r="AD1" s="395"/>
-      <c r="AE1" s="395"/>
-      <c r="AF1" s="395"/>
-      <c r="AG1" s="401"/>
-      <c r="AH1" s="396"/>
-      <c r="AI1" s="401"/>
-      <c r="AJ1" s="401"/>
-      <c r="AK1" s="396"/>
-      <c r="AL1" s="401"/>
-      <c r="AM1" s="401"/>
-      <c r="AN1" s="401"/>
-      <c r="AO1" s="401"/>
+      <c r="B1" s="407"/>
+      <c r="C1" s="408"/>
+      <c r="D1" s="408"/>
+      <c r="E1" s="409"/>
+      <c r="F1" s="409"/>
+      <c r="G1" s="409"/>
+      <c r="H1" s="401"/>
+      <c r="I1" s="401"/>
+      <c r="J1" s="401"/>
+      <c r="K1" s="402"/>
+      <c r="L1" s="401"/>
+      <c r="M1" s="401"/>
+      <c r="N1" s="410"/>
+      <c r="O1" s="410"/>
+      <c r="P1" s="410"/>
+      <c r="Q1" s="410"/>
+      <c r="R1" s="410"/>
+      <c r="S1" s="410"/>
+      <c r="T1" s="410"/>
+      <c r="U1" s="410"/>
+      <c r="V1" s="410"/>
+      <c r="W1" s="410"/>
+      <c r="X1" s="410"/>
+      <c r="Y1" s="410"/>
+      <c r="Z1" s="410"/>
+      <c r="AA1" s="410"/>
+      <c r="AB1" s="410"/>
+      <c r="AC1" s="410"/>
+      <c r="AD1" s="410"/>
+      <c r="AE1" s="410"/>
+      <c r="AF1" s="410"/>
+      <c r="AG1" s="392"/>
+      <c r="AH1" s="402"/>
+      <c r="AI1" s="392"/>
+      <c r="AJ1" s="392"/>
+      <c r="AK1" s="402"/>
+      <c r="AL1" s="392"/>
+      <c r="AM1" s="392"/>
+      <c r="AN1" s="392"/>
+      <c r="AO1" s="392"/>
       <c r="AP1" s="113"/>
       <c r="AQ1" s="341"/>
       <c r="AR1" s="341"/>
@@ -13253,12 +13230,12 @@
       <c r="F3" s="9"/>
       <c r="G3" s="9"/>
       <c r="H3" s="23"/>
-      <c r="I3" s="412" t="s">
-        <v>0</v>
-      </c>
-      <c r="J3" s="400"/>
-      <c r="K3" s="396"/>
-      <c r="L3" s="400"/>
+      <c r="I3" s="400" t="s">
+        <v>0</v>
+      </c>
+      <c r="J3" s="401"/>
+      <c r="K3" s="402"/>
+      <c r="L3" s="401"/>
       <c r="V3" s="8"/>
       <c r="W3" s="8"/>
       <c r="X3" s="8"/>
@@ -13400,11 +13377,11 @@
       <c r="AM7" s="8"/>
       <c r="AN7" s="8"/>
       <c r="AO7" s="8"/>
-      <c r="AT7" s="391" t="s">
+      <c r="AT7" s="406" t="s">
         <v>5</v>
       </c>
-      <c r="AU7" s="392"/>
-      <c r="AV7" s="393"/>
+      <c r="AU7" s="404"/>
+      <c r="AV7" s="405"/>
       <c r="AW7" s="344"/>
       <c r="AY7" s="345" t="s">
         <v>6</v>
@@ -17748,20 +17725,20 @@
       <c r="T62" s="46"/>
       <c r="U62" s="46"/>
       <c r="V62" s="46"/>
-      <c r="W62" s="402" t="s">
+      <c r="W62" s="403" t="s">
         <v>55</v>
       </c>
-      <c r="X62" s="392"/>
-      <c r="Y62" s="393"/>
+      <c r="X62" s="404"/>
+      <c r="Y62" s="405"/>
       <c r="Z62" s="46"/>
       <c r="AA62" s="8"/>
-      <c r="AB62" s="402" t="s">
+      <c r="AB62" s="403" t="s">
         <v>56</v>
       </c>
-      <c r="AC62" s="392"/>
-      <c r="AD62" s="392"/>
-      <c r="AE62" s="392"/>
-      <c r="AF62" s="393"/>
+      <c r="AC62" s="404"/>
+      <c r="AD62" s="404"/>
+      <c r="AE62" s="404"/>
+      <c r="AF62" s="405"/>
       <c r="AG62" s="8"/>
       <c r="AY62" s="357"/>
     </row>
@@ -18804,11 +18781,11 @@
     <mergeCell ref="B1:AO1"/>
   </mergeCells>
   <conditionalFormatting sqref="K34:K44">
-    <cfRule type="cellIs" dxfId="198" priority="476" operator="equal">
+    <cfRule type="cellIs" dxfId="198" priority="475" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="197" priority="476" operator="equal">
       <formula>"YES"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="197" priority="475" operator="equal">
-      <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K48:K54">
@@ -18820,31 +18797,31 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W63">
-    <cfRule type="cellIs" dxfId="194" priority="497" operator="equal">
-      <formula>"YES"</formula>
+    <cfRule type="cellIs" dxfId="194" priority="495" operator="equal">
+      <formula>"NO-OOS"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="193" priority="496" operator="equal">
       <formula>"NO-CO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="192" priority="495" operator="equal">
-      <formula>"NO-OOS"</formula>
+    <cfRule type="cellIs" dxfId="192" priority="497" operator="equal">
+      <formula>"YES"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="191" priority="498" operator="equal">
       <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB63">
-    <cfRule type="cellIs" dxfId="190" priority="493" operator="equal">
-      <formula>"NO"</formula>
+    <cfRule type="cellIs" dxfId="190" priority="490" operator="equal">
+      <formula>"NO-OOS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="189" priority="492" operator="equal">
+    <cfRule type="cellIs" dxfId="189" priority="491" operator="equal">
+      <formula>"NO-CO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="188" priority="492" operator="equal">
       <formula>"YES"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="188" priority="490" operator="equal">
-      <formula>"NO-OOS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="187" priority="491" operator="equal">
-      <formula>"NO-CO"</formula>
+    <cfRule type="cellIs" dxfId="187" priority="493" operator="equal">
+      <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AG9:AG54">
@@ -18893,11 +18870,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AK23 AN23">
-    <cfRule type="cellIs" dxfId="175" priority="529" operator="equal">
+    <cfRule type="cellIs" dxfId="175" priority="528" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="174" priority="529" operator="equal">
       <formula>"YES"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="174" priority="528" operator="equal">
-      <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AK25 AN25">
@@ -18949,19 +18926,19 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AK45:AK54 AN45:AN54">
-    <cfRule type="cellIs" dxfId="161" priority="125" operator="equal">
+    <cfRule type="cellIs" dxfId="161" priority="124" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="160" priority="125" operator="equal">
       <formula>"YES"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="160" priority="124" operator="equal">
-      <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AK9:AN10 AK27:AN27">
-    <cfRule type="cellIs" dxfId="159" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="159" priority="3" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="158" priority="4" operator="equal">
       <formula>"YES"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="158" priority="3" operator="equal">
-      <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AL11:AM26 B55:G55">
@@ -18989,11 +18966,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AL43:AN43">
-    <cfRule type="cellIs" dxfId="151" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="151" priority="5" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="150" priority="6" operator="equal">
       <formula>"YES"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="150" priority="5" operator="equal">
-      <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AN11:AN14">
@@ -19005,11 +18982,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AQ9:AQ54">
-    <cfRule type="cellIs" dxfId="147" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="147" priority="1" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="146" priority="2" operator="equal">
       <formula>"YES"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="146" priority="1" operator="equal">
-      <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations disablePrompts="1" count="1">
@@ -19059,33 +19036,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="397"/>
-      <c r="C1" s="413"/>
-      <c r="D1" s="396"/>
-      <c r="E1" s="400"/>
-      <c r="F1" s="400"/>
-      <c r="G1" s="414"/>
-      <c r="H1" s="414"/>
-      <c r="I1" s="414"/>
-      <c r="J1" s="414"/>
-      <c r="K1" s="414"/>
-      <c r="L1" s="414"/>
-      <c r="M1" s="415"/>
-      <c r="N1" s="415"/>
-      <c r="O1" s="416"/>
-      <c r="P1" s="396"/>
-      <c r="Q1" s="396"/>
-      <c r="R1" s="396"/>
-      <c r="S1" s="396"/>
-      <c r="T1" s="417"/>
-      <c r="U1" s="417"/>
-      <c r="V1" s="396"/>
-      <c r="W1" s="396"/>
-      <c r="X1" s="396"/>
-      <c r="Y1" s="396"/>
-      <c r="Z1" s="417"/>
-      <c r="AA1" s="401"/>
-      <c r="AB1" s="417"/>
+      <c r="B1" s="407"/>
+      <c r="C1" s="411"/>
+      <c r="D1" s="402"/>
+      <c r="E1" s="401"/>
+      <c r="F1" s="401"/>
+      <c r="G1" s="412"/>
+      <c r="H1" s="412"/>
+      <c r="I1" s="412"/>
+      <c r="J1" s="412"/>
+      <c r="K1" s="412"/>
+      <c r="L1" s="412"/>
+      <c r="M1" s="413"/>
+      <c r="N1" s="413"/>
+      <c r="O1" s="414"/>
+      <c r="P1" s="402"/>
+      <c r="Q1" s="402"/>
+      <c r="R1" s="402"/>
+      <c r="S1" s="402"/>
+      <c r="T1" s="415"/>
+      <c r="U1" s="415"/>
+      <c r="V1" s="402"/>
+      <c r="W1" s="402"/>
+      <c r="X1" s="402"/>
+      <c r="Y1" s="402"/>
+      <c r="Z1" s="415"/>
+      <c r="AA1" s="392"/>
+      <c r="AB1" s="415"/>
       <c r="AC1" s="113"/>
       <c r="AD1" s="113"/>
       <c r="AE1" s="113"/>
@@ -19202,7 +19179,7 @@
       <c r="C7" s="101"/>
       <c r="D7" s="101"/>
       <c r="F7" s="27" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="K7" s="119"/>
       <c r="P7" s="119"/>
@@ -19223,31 +19200,31 @@
     </row>
     <row r="8" spans="1:31" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="B8" s="285" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="277" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="D8" s="284" t="s">
         <v>52</v>
       </c>
       <c r="E8" s="287" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="F8" s="279" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="G8" s="288" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="H8" s="288" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="I8" s="288" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="J8" s="288" t="s">
         <v>103</v>
@@ -19256,7 +19233,7 @@
         <v>61</v>
       </c>
       <c r="L8" s="288" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="M8" s="290" t="s">
         <v>14</v>
@@ -19268,25 +19245,25 @@
         <v>16</v>
       </c>
       <c r="P8" s="315" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="Q8" s="315" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="R8" s="315" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="S8" s="315" t="s">
         <v>39</v>
       </c>
       <c r="T8" s="315" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="U8" s="315" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="V8" s="315" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="W8" s="315" t="s">
         <v>168</v>
@@ -19298,7 +19275,7 @@
         <v>45</v>
       </c>
       <c r="Z8" s="315" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="AA8" s="315" t="s">
         <v>41</v>
@@ -20810,16 +20787,16 @@
       <c r="F43" s="28"/>
       <c r="G43" s="291"/>
       <c r="H43" s="291" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="I43" s="291" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="J43" s="291" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="K43" s="291" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="L43" s="72">
         <f>SUM(L9:L39)</f>
@@ -20851,11 +20828,11 @@
       <c r="F47" s="128"/>
       <c r="G47" s="129"/>
       <c r="H47" s="8"/>
-      <c r="J47" s="402" t="s">
+      <c r="J47" s="403" t="s">
         <v>56</v>
       </c>
-      <c r="K47" s="392"/>
-      <c r="L47" s="393"/>
+      <c r="K47" s="404"/>
+      <c r="L47" s="405"/>
       <c r="M47" s="8"/>
       <c r="N47" s="8"/>
       <c r="O47" s="8"/>
@@ -21141,27 +21118,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="397"/>
-      <c r="B1" s="398"/>
-      <c r="C1" s="398"/>
-      <c r="D1" s="398"/>
-      <c r="E1" s="399"/>
-      <c r="F1" s="400"/>
-      <c r="G1" s="400"/>
-      <c r="H1" s="401"/>
-      <c r="I1" s="396"/>
-      <c r="J1" s="399"/>
-      <c r="K1" s="396"/>
-      <c r="L1" s="396"/>
-      <c r="M1" s="395"/>
-      <c r="N1" s="395"/>
-      <c r="O1" s="395"/>
-      <c r="P1" s="395"/>
-      <c r="Q1" s="395"/>
-      <c r="R1" s="395"/>
-      <c r="S1" s="395"/>
-      <c r="T1" s="395"/>
-      <c r="U1" s="395"/>
+      <c r="A1" s="407"/>
+      <c r="B1" s="408"/>
+      <c r="C1" s="408"/>
+      <c r="D1" s="408"/>
+      <c r="E1" s="409"/>
+      <c r="F1" s="401"/>
+      <c r="G1" s="401"/>
+      <c r="H1" s="392"/>
+      <c r="I1" s="402"/>
+      <c r="J1" s="409"/>
+      <c r="K1" s="402"/>
+      <c r="L1" s="402"/>
+      <c r="M1" s="410"/>
+      <c r="N1" s="410"/>
+      <c r="O1" s="410"/>
+      <c r="P1" s="410"/>
+      <c r="Q1" s="410"/>
+      <c r="R1" s="410"/>
+      <c r="S1" s="410"/>
+      <c r="T1" s="410"/>
+      <c r="U1" s="410"/>
       <c r="V1" s="113"/>
       <c r="W1" s="113"/>
       <c r="X1" s="113"/>
@@ -21229,12 +21206,12 @@
       <c r="Q3" s="222"/>
       <c r="R3" s="222"/>
       <c r="S3" s="222"/>
-      <c r="V3" s="394" t="s">
-        <v>227</v>
-      </c>
-      <c r="W3" s="395"/>
-      <c r="X3" s="396"/>
-      <c r="Y3" s="396"/>
+      <c r="V3" s="416" t="s">
+        <v>220</v>
+      </c>
+      <c r="W3" s="410"/>
+      <c r="X3" s="402"/>
+      <c r="Y3" s="402"/>
       <c r="AD3" s="32"/>
       <c r="AE3" s="32"/>
       <c r="AI3" s="32"/>
@@ -21250,12 +21227,12 @@
       <c r="J4" s="112"/>
       <c r="K4" s="112"/>
       <c r="L4" s="112"/>
-      <c r="V4" s="394" t="s">
-        <v>228</v>
-      </c>
-      <c r="W4" s="395"/>
-      <c r="X4" s="396"/>
-      <c r="Y4" s="396"/>
+      <c r="V4" s="416" t="s">
+        <v>221</v>
+      </c>
+      <c r="W4" s="410"/>
+      <c r="X4" s="402"/>
+      <c r="Y4" s="402"/>
       <c r="Z4" s="5"/>
       <c r="AA4" s="173"/>
       <c r="AC4" s="4"/>
@@ -21280,7 +21257,7 @@
       <c r="K5" s="112"/>
       <c r="L5" s="112"/>
       <c r="Q5" s="174" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="R5" s="174"/>
       <c r="S5" s="174"/>
@@ -21330,36 +21307,36 @@
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.3">
       <c r="M7" s="176" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="N7" s="176"/>
       <c r="O7" s="176" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="P7" s="176"/>
       <c r="Q7" s="176" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="S7" s="176" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="T7" s="176" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="W7" s="176" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="AB7" s="176" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="AI7" s="176" t="s">
-        <v>230</v>
-      </c>
-      <c r="AK7" s="391" t="s">
+        <v>223</v>
+      </c>
+      <c r="AK7" s="406" t="s">
         <v>5</v>
       </c>
-      <c r="AL7" s="392"/>
-      <c r="AM7" s="393"/>
+      <c r="AL7" s="404"/>
+      <c r="AM7" s="405"/>
       <c r="AP7" s="345" t="s">
         <v>6</v>
       </c>
@@ -21369,10 +21346,10 @@
         <v>7</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="E8" s="79" t="s">
         <v>52</v>
@@ -21381,46 +21358,46 @@
         <v>11</v>
       </c>
       <c r="G8" s="254" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J8" s="12" t="s">
         <v>16</v>
       </c>
       <c r="K8" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="L8" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="M8" s="44" t="s">
+        <v>229</v>
+      </c>
+      <c r="N8" s="44" t="s">
+        <v>230</v>
+      </c>
+      <c r="O8" s="48" t="s">
+        <v>209</v>
+      </c>
+      <c r="P8" s="48" t="s">
+        <v>210</v>
+      </c>
+      <c r="Q8" s="44" t="s">
+        <v>231</v>
+      </c>
+      <c r="R8" s="44" t="s">
+        <v>232</v>
+      </c>
+      <c r="S8" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="T8" s="44" t="s">
         <v>234</v>
-      </c>
-      <c r="L8" s="12" t="s">
-        <v>235</v>
-      </c>
-      <c r="M8" s="44" t="s">
-        <v>236</v>
-      </c>
-      <c r="N8" s="44" t="s">
-        <v>237</v>
-      </c>
-      <c r="O8" s="48" t="s">
-        <v>216</v>
-      </c>
-      <c r="P8" s="48" t="s">
-        <v>217</v>
-      </c>
-      <c r="Q8" s="44" t="s">
-        <v>238</v>
-      </c>
-      <c r="R8" s="44" t="s">
-        <v>239</v>
-      </c>
-      <c r="S8" s="44" t="s">
-        <v>240</v>
-      </c>
-      <c r="T8" s="44" t="s">
-        <v>241</v>
       </c>
       <c r="U8" s="44" t="s">
         <v>32</v>
@@ -21432,10 +21409,10 @@
         <v>34</v>
       </c>
       <c r="X8" s="12" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="Y8" s="12" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="Z8" s="12" t="s">
         <v>38</v>
@@ -21444,16 +21421,16 @@
         <v>39</v>
       </c>
       <c r="AB8" s="12" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="AC8" s="79" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="AD8" s="12" t="s">
         <v>41</v>
       </c>
       <c r="AE8" s="12" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="AF8" s="12" t="s">
         <v>43</v>
@@ -21471,7 +21448,7 @@
         <v>49</v>
       </c>
       <c r="AL8" s="350" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="AM8" s="350" t="s">
         <v>51</v>
@@ -23849,17 +23826,17 @@
         <v>52</v>
       </c>
       <c r="F45" s="167" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="G45" s="167"/>
       <c r="H45" s="167" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="I45" s="167" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="J45" s="167" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="K45" s="167" t="s">
         <v>32</v>
@@ -23914,19 +23891,19 @@
       </c>
       <c r="M47" s="8"/>
       <c r="N47" s="8"/>
-      <c r="O47" s="402" t="s">
+      <c r="O47" s="403" t="s">
         <v>55</v>
       </c>
-      <c r="P47" s="392"/>
-      <c r="Q47" s="392"/>
-      <c r="R47" s="393"/>
+      <c r="P47" s="404"/>
+      <c r="Q47" s="404"/>
+      <c r="R47" s="405"/>
       <c r="S47" s="8"/>
       <c r="T47" s="46"/>
-      <c r="U47" s="403" t="s">
+      <c r="U47" s="417" t="s">
         <v>56</v>
       </c>
-      <c r="V47" s="392"/>
-      <c r="W47" s="393"/>
+      <c r="V47" s="404"/>
+      <c r="W47" s="405"/>
       <c r="X47" s="187"/>
       <c r="Y47" s="188"/>
       <c r="Z47" s="188"/>
@@ -23967,7 +23944,7 @@
         <v>59</v>
       </c>
       <c r="R48" s="190" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="S48" s="46"/>
       <c r="T48" s="89"/>
@@ -24681,11 +24658,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J40:L40">
-    <cfRule type="cellIs" dxfId="123" priority="475" operator="equal">
+    <cfRule type="cellIs" dxfId="123" priority="474" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="122" priority="475" operator="equal">
       <formula>"YES"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="122" priority="474" operator="equal">
-      <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L9:L39">
@@ -24697,11 +24674,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O48">
-    <cfRule type="cellIs" dxfId="119" priority="487" operator="equal">
+    <cfRule type="cellIs" dxfId="119" priority="486" operator="equal">
+      <formula>"NO-OOS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="118" priority="487" operator="equal">
       <formula>"NO-CO"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="118" priority="486" operator="equal">
-      <formula>"NO-OOS"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="117" priority="488" operator="equal">
       <formula>"YES"</formula>
@@ -24711,25 +24688,25 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U48">
-    <cfRule type="cellIs" dxfId="115" priority="483" operator="equal">
-      <formula>"YES"</formula>
+    <cfRule type="cellIs" dxfId="115" priority="481" operator="equal">
+      <formula>"NO-OOS"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="114" priority="482" operator="equal">
       <formula>"NO-CO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="113" priority="481" operator="equal">
-      <formula>"NO-OOS"</formula>
+    <cfRule type="cellIs" dxfId="113" priority="483" operator="equal">
+      <formula>"YES"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="112" priority="484" operator="equal">
       <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z9:Z39">
-    <cfRule type="cellIs" dxfId="111" priority="295" operator="equal">
+    <cfRule type="cellIs" dxfId="111" priority="294" operator="equal">
+      <formula>"N/A"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="110" priority="295" operator="equal">
       <formula>"YES"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="110" priority="294" operator="equal">
-      <formula>"N/A"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="109" priority="296" operator="equal">
       <formula>"NO"</formula>
@@ -24749,11 +24726,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC60">
-    <cfRule type="cellIs" dxfId="105" priority="458" operator="equal">
+    <cfRule type="cellIs" dxfId="105" priority="456" operator="equal">
+      <formula>"N/A"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="104" priority="458" operator="equal">
       <formula>"NO"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="104" priority="456" operator="equal">
-      <formula>"N/A"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC60:AH60">
@@ -24780,11 +24757,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD60">
-    <cfRule type="cellIs" dxfId="98" priority="461" operator="equal">
+    <cfRule type="cellIs" dxfId="98" priority="459" operator="equal">
+      <formula>"NO-OOS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="97" priority="461" operator="equal">
       <formula>"NO-TX"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="97" priority="459" operator="equal">
-      <formula>"NO-OOS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE16:AE25">
@@ -24804,19 +24781,19 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE10:AG10">
-    <cfRule type="cellIs" dxfId="92" priority="269" operator="equal">
+    <cfRule type="cellIs" dxfId="92" priority="268" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="91" priority="269" operator="equal">
       <formula>"YES"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="91" priority="268" operator="equal">
-      <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE14:AG14">
-    <cfRule type="cellIs" dxfId="90" priority="273" operator="equal">
+    <cfRule type="cellIs" dxfId="90" priority="272" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="89" priority="273" operator="equal">
       <formula>"YES"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="89" priority="272" operator="equal">
-      <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE26:AG38">
@@ -24836,11 +24813,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE11:AH11 AE12:AG12 AE13:AH13">
-    <cfRule type="cellIs" dxfId="84" priority="285" operator="equal">
+    <cfRule type="cellIs" dxfId="84" priority="284" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="83" priority="285" operator="equal">
       <formula>"YES"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="83" priority="284" operator="equal">
-      <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE15:AH15">
@@ -24852,11 +24829,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE38:AH40">
-    <cfRule type="cellIs" dxfId="80" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="80" priority="16" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="79" priority="17" operator="equal">
       <formula>"YES"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="79" priority="16" operator="equal">
-      <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE60:AH60">
@@ -24865,35 +24842,35 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF16:AG16">
-    <cfRule type="cellIs" dxfId="77" priority="271" operator="equal">
+    <cfRule type="cellIs" dxfId="77" priority="270" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="76" priority="271" operator="equal">
       <formula>"YES"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="76" priority="270" operator="equal">
-      <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF23:AG25">
-    <cfRule type="cellIs" dxfId="75" priority="66" operator="equal">
+    <cfRule type="cellIs" dxfId="75" priority="65" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="74" priority="66" operator="equal">
       <formula>"YES"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="74" priority="65" operator="equal">
-      <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF17:AH22">
-    <cfRule type="cellIs" dxfId="73" priority="279" operator="equal">
+    <cfRule type="cellIs" dxfId="73" priority="278" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="72" priority="279" operator="equal">
       <formula>"YES"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="72" priority="278" operator="equal">
-      <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AH9:AH38">
-    <cfRule type="cellIs" dxfId="71" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="71" priority="20" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="70" priority="21" operator="equal">
       <formula>"YES"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="70" priority="20" operator="equal">
-      <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -25075,7 +25052,7 @@
         <v>7</v>
       </c>
       <c r="C7" s="79" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="D7" s="12" t="s">
         <v>52</v>
@@ -25087,13 +25064,13 @@
         <v>12</v>
       </c>
       <c r="G7" s="48" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="H7" s="48" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="I7" s="48" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="J7" s="48" t="s">
         <v>103</v>
@@ -25102,10 +25079,10 @@
         <v>61</v>
       </c>
       <c r="L7" s="48" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="M7" s="67" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="N7" s="204" t="s">
         <v>15</v>
@@ -25114,25 +25091,25 @@
         <v>16</v>
       </c>
       <c r="P7" s="12" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="Q7" s="12" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="R7" s="12" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="S7" s="12" t="s">
         <v>39</v>
       </c>
       <c r="T7" s="12" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="U7" s="12" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="V7" s="12" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="W7" s="12" t="s">
         <v>168</v>
@@ -25144,7 +25121,7 @@
         <v>45</v>
       </c>
       <c r="Z7" s="12" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="AA7" s="12" t="s">
         <v>41</v>
@@ -26662,17 +26639,17 @@
       <c r="AA45" s="32"/>
     </row>
     <row r="46" spans="2:28" x14ac:dyDescent="0.3">
-      <c r="D46" s="402" t="s">
+      <c r="D46" s="403" t="s">
         <v>55</v>
       </c>
-      <c r="E46" s="392"/>
-      <c r="F46" s="393"/>
+      <c r="E46" s="404"/>
+      <c r="F46" s="405"/>
       <c r="G46" s="8"/>
-      <c r="I46" s="402" t="s">
+      <c r="I46" s="403" t="s">
         <v>56</v>
       </c>
-      <c r="J46" s="392"/>
-      <c r="K46" s="393"/>
+      <c r="J46" s="404"/>
+      <c r="K46" s="405"/>
       <c r="L46" s="8"/>
       <c r="M46" s="8"/>
       <c r="N46" s="8"/>
@@ -26948,29 +26925,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="397"/>
-      <c r="C1" s="413"/>
-      <c r="D1" s="396"/>
-      <c r="E1" s="400"/>
-      <c r="F1" s="414"/>
-      <c r="G1" s="414"/>
-      <c r="H1" s="414"/>
-      <c r="I1" s="415"/>
-      <c r="J1" s="396"/>
-      <c r="K1" s="396"/>
-      <c r="L1" s="417"/>
-      <c r="M1" s="396"/>
-      <c r="N1" s="396"/>
-      <c r="O1" s="417"/>
-      <c r="P1" s="417"/>
-      <c r="Q1" s="396"/>
-      <c r="R1" s="396"/>
-      <c r="S1" s="396"/>
-      <c r="T1" s="396"/>
-      <c r="U1" s="417"/>
-      <c r="V1" s="401"/>
-      <c r="W1" s="417"/>
-      <c r="X1" s="401"/>
+      <c r="B1" s="407"/>
+      <c r="C1" s="411"/>
+      <c r="D1" s="402"/>
+      <c r="E1" s="401"/>
+      <c r="F1" s="412"/>
+      <c r="G1" s="412"/>
+      <c r="H1" s="412"/>
+      <c r="I1" s="413"/>
+      <c r="J1" s="402"/>
+      <c r="K1" s="402"/>
+      <c r="L1" s="415"/>
+      <c r="M1" s="402"/>
+      <c r="N1" s="402"/>
+      <c r="O1" s="415"/>
+      <c r="P1" s="415"/>
+      <c r="Q1" s="402"/>
+      <c r="R1" s="402"/>
+      <c r="S1" s="402"/>
+      <c r="T1" s="402"/>
+      <c r="U1" s="415"/>
+      <c r="V1" s="392"/>
+      <c r="W1" s="415"/>
+      <c r="X1" s="392"/>
     </row>
     <row r="2" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="113"/>
@@ -27083,7 +27060,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="272" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="D8" s="274" t="s">
         <v>52</v>
@@ -27092,40 +27069,40 @@
         <v>11</v>
       </c>
       <c r="F8" s="292" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="G8" s="369" t="s">
         <v>61</v>
       </c>
       <c r="H8" s="292" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="I8" s="293" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="J8" s="274" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="K8" s="274" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="L8" s="274" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="M8" s="274" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="N8" s="274" t="s">
         <v>39</v>
       </c>
       <c r="O8" s="274" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="P8" s="274" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="Q8" s="274" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="R8" s="274" t="s">
         <v>168</v>
@@ -27137,7 +27114,7 @@
         <v>45</v>
       </c>
       <c r="U8" s="274" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="V8" s="274" t="s">
         <v>41</v>
@@ -29275,7 +29252,7 @@
       <c r="E92" s="28"/>
       <c r="F92" s="291"/>
       <c r="G92" s="295" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="H92" s="72">
         <f>SUM(H9:H88)</f>
@@ -29299,17 +29276,17 @@
       <c r="M93" s="14"/>
     </row>
     <row r="96" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="D96" s="402" t="s">
+      <c r="D96" s="403" t="s">
         <v>55</v>
       </c>
-      <c r="E96" s="392"/>
-      <c r="F96" s="393"/>
+      <c r="E96" s="404"/>
+      <c r="F96" s="405"/>
       <c r="G96" s="8"/>
-      <c r="I96" s="402" t="s">
+      <c r="I96" s="403" t="s">
         <v>56</v>
       </c>
-      <c r="J96" s="392"/>
-      <c r="K96" s="393"/>
+      <c r="J96" s="404"/>
+      <c r="K96" s="405"/>
       <c r="L96" s="8"/>
     </row>
     <row r="97" spans="4:12" x14ac:dyDescent="0.3">
@@ -29431,7 +29408,7 @@
     </row>
     <row r="106" spans="4:12" x14ac:dyDescent="0.3">
       <c r="G106" s="162" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="H106" s="162" t="s">
         <v>32</v>
@@ -29445,7 +29422,7 @@
     </row>
     <row r="107" spans="4:12" x14ac:dyDescent="0.3">
       <c r="G107" s="46" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="H107" s="46">
         <f>SUMIF($J$9:$J$88,G107,$F$9:$F$88)</f>
@@ -29462,7 +29439,7 @@
     </row>
     <row r="108" spans="4:12" x14ac:dyDescent="0.3">
       <c r="G108" s="46" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="H108" s="46">
         <f>SUMIF($J$9:$J$88,G108,$F$9:$F$88)</f>
@@ -29479,7 +29456,7 @@
     </row>
     <row r="109" spans="4:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G109" s="97" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="H109" s="97">
         <f>SUMIF($J$9:$J$88,G109,$F$9:$F$88)</f>
@@ -29645,17 +29622,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f4e7d37e-1dcc-4436-a729-076bff741eab">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="7ff3518b-2e3d-4dfb-a834-48e552d5b5bf" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100504A511723502843AC0584E68EC60535" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fbd80a4f17478eeb58df59f7f6ca8f1e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f4e7d37e-1dcc-4436-a729-076bff741eab" xmlns:ns3="7ff3518b-2e3d-4dfb-a834-48e552d5b5bf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="88c3fc8cee6a1370bae988e1d6c9e850" ns2:_="" ns3:_="">
     <xsd:import namespace="f4e7d37e-1dcc-4436-a729-076bff741eab"/>
@@ -29850,6 +29816,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f4e7d37e-1dcc-4436-a729-076bff741eab">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="7ff3518b-2e3d-4dfb-a834-48e552d5b5bf" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7896FE09-375C-4B80-B12E-A86A22AFA945}">
   <ds:schemaRefs>
@@ -29859,17 +29836,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{52B44F4C-5208-463C-B02B-93FE2A2E7C51}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="f4e7d37e-1dcc-4436-a729-076bff741eab"/>
-    <ds:schemaRef ds:uri="7ff3518b-2e3d-4dfb-a834-48e552d5b5bf"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B400FA9-B915-4F5E-9F2F-389D7B15AAF3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -29886,4 +29852,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{52B44F4C-5208-463C-B02B-93FE2A2E7C51}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f4e7d37e-1dcc-4436-a729-076bff741eab"/>
+    <ds:schemaRef ds:uri="7ff3518b-2e3d-4dfb-a834-48e552d5b5bf"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>